<commit_message>
chore(predeploy): limpa arquivos temporários e valida build
</commit_message>
<xml_diff>
--- a/public/template-diario-de-campo.xlsx
+++ b/public/template-diario-de-campo.xlsx
@@ -24,7 +24,7 @@
     <t>Data * (AAAA-MM-DD)</t>
   </si>
   <si>
-    <t>Responsável *</t>
+    <t>Equipe *</t>
   </si>
   <si>
     <t>Local / Reservatório *</t>
@@ -261,7 +261,7 @@
     <t xml:space="preserve">  • Data — formato AAAA-MM-DD (ex: 2026-05-20)</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Responsável — nome completo do técnico de campo</t>
+    <t xml:space="preserve">  • Equipe — nome completo do técnico ou equipe de campo</t>
   </si>
   <si>
     <t xml:space="preserve">  • Local / Reservatório — nome do ponto de coleta</t>
@@ -321,7 +321,7 @@
     <t xml:space="preserve">  • O separador para múltiplos valores em Atividades e Condições é ponto e vírgula (;)</t>
   </si>
   <si>
-    <t xml:space="preserve">  • Registros duplicados (mesmo Local + Data + Campanha + Responsável) podem ser re-importados</t>
+    <t xml:space="preserve">  • Registros duplicados (mesmo Local + Data + Campanha + Equipe) podem ser re-importados</t>
   </si>
 </sst>
 </file>

</xml_diff>